<commit_message>
fix: refactor objective function to restore gradient landscape and rerun
</commit_message>
<xml_diff>
--- a/STITP_Experimental_Data.xlsx
+++ b/STITP_Experimental_Data.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Convergence_Curves" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,28 +469,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.06008811298006956</v>
+        <v>0.07988574344794946</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06015181047371371</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08832228105995965</v>
+        <v>0.1082951519718369</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06686094557612325</v>
+        <v>0.07903532404589769</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06489743309619406</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06030710886177843</v>
+        <v>0.0792070809884846</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06282998666125421</v>
+        <v>0.07904080983021997</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06677083062764706</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="3">
@@ -499,28 +498,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.06008811298006956</v>
+        <v>0.07988574344794946</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06015181047371371</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D3" t="n">
-        <v>0.06087014090589951</v>
+        <v>0.1082951519718369</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06486969731646747</v>
+        <v>0.07903532404589769</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0600906111744703</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G3" t="n">
-        <v>0.06012321937410896</v>
+        <v>0.0792070809884846</v>
       </c>
       <c r="H3" t="n">
-        <v>0.06092064457847277</v>
+        <v>0.07904080983021997</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0652664260117172</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="4">
@@ -528,28 +527,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.06008811298006956</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06015181047371371</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06015130495878051</v>
+        <v>0.08308718263728132</v>
       </c>
       <c r="E4" t="n">
-        <v>0.06486969731646747</v>
+        <v>0.07903532404589769</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0600906111744703</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G4" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.0792070809884846</v>
       </c>
       <c r="H4" t="n">
-        <v>0.06014235314343052</v>
+        <v>0.07890327709690365</v>
       </c>
       <c r="I4" t="n">
-        <v>0.06127992723482242</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="5">
@@ -557,28 +556,28 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.06008811298006956</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C5" t="n">
-        <v>0.06015181047371371</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D5" t="n">
-        <v>0.06015130495878051</v>
+        <v>0.08239146057829372</v>
       </c>
       <c r="E5" t="n">
-        <v>0.06486969731646747</v>
+        <v>0.07903532404589769</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0600906111744703</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.0792070809884846</v>
       </c>
       <c r="H5" t="n">
-        <v>0.06013529794388074</v>
+        <v>0.07890248734805461</v>
       </c>
       <c r="I5" t="n">
-        <v>0.06057461590353382</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="6">
@@ -586,28 +585,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C6" t="n">
-        <v>0.06015181047371371</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06015130495878051</v>
+        <v>0.0797357590674346</v>
       </c>
       <c r="E6" t="n">
-        <v>0.06372358900569154</v>
+        <v>0.07890633814757395</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0600906111744703</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G6" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.0792070809884846</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06009384270521864</v>
+        <v>0.07890248734805461</v>
       </c>
       <c r="I6" t="n">
-        <v>0.06057461590353382</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="7">
@@ -615,28 +614,28 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C7" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D7" t="n">
-        <v>0.06015130495878051</v>
+        <v>0.07967650429838982</v>
       </c>
       <c r="E7" t="n">
-        <v>0.06372358900569154</v>
+        <v>0.07890633814757395</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0600906111744703</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G7" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.0790328255063954</v>
       </c>
       <c r="H7" t="n">
-        <v>0.06009197518821138</v>
+        <v>0.07890248734805461</v>
       </c>
       <c r="I7" t="n">
-        <v>0.06057461590353382</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="8">
@@ -644,28 +643,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C8" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06009534767992612</v>
+        <v>0.0791281190919845</v>
       </c>
       <c r="E8" t="n">
-        <v>0.06372358900569154</v>
+        <v>0.07890633814757395</v>
       </c>
       <c r="F8" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G8" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.0790328255063954</v>
       </c>
       <c r="H8" t="n">
-        <v>0.06009197518821138</v>
+        <v>0.07890235522774873</v>
       </c>
       <c r="I8" t="n">
-        <v>0.06057461590353382</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="9">
@@ -673,28 +672,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C9" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D9" t="n">
-        <v>0.06009534767992612</v>
+        <v>0.0791281190919845</v>
       </c>
       <c r="E9" t="n">
-        <v>0.06372358900569154</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F9" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G9" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.07890257930464979</v>
       </c>
       <c r="H9" t="n">
-        <v>0.06008821433568048</v>
+        <v>0.07890235522774873</v>
       </c>
       <c r="I9" t="n">
-        <v>0.06017217680421726</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="10">
@@ -702,28 +701,28 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C10" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D10" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0791281190919845</v>
       </c>
       <c r="E10" t="n">
-        <v>0.06372358900569154</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F10" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G10" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.07890257930464979</v>
       </c>
       <c r="H10" t="n">
-        <v>0.06008821433568048</v>
+        <v>0.07890235522774873</v>
       </c>
       <c r="I10" t="n">
-        <v>0.06017217680421726</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="11">
@@ -731,28 +730,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C11" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D11" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0791281190919845</v>
       </c>
       <c r="E11" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F11" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G11" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H11" t="n">
-        <v>0.06008821433568048</v>
+        <v>0.07890235522774873</v>
       </c>
       <c r="I11" t="n">
-        <v>0.06017217680421726</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="12">
@@ -760,28 +759,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C12" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D12" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E12" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F12" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G12" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H12" t="n">
-        <v>0.06008805864859965</v>
+        <v>0.0789023330096072</v>
       </c>
       <c r="I12" t="n">
-        <v>0.06017217680421726</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="13">
@@ -789,28 +788,28 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>0.06008792174991699</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D13" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E13" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F13" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G13" t="n">
-        <v>0.06009051696973755</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H13" t="n">
-        <v>0.06008805310291566</v>
+        <v>0.07890232123221913</v>
       </c>
       <c r="I13" t="n">
-        <v>0.06017217680421726</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="14">
@@ -818,28 +817,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C14" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D14" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E14" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F14" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G14" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H14" t="n">
-        <v>0.06008794482067521</v>
+        <v>0.07890232123221913</v>
       </c>
       <c r="I14" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="15">
@@ -847,28 +846,28 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D15" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E15" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F15" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G15" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H15" t="n">
-        <v>0.06008794482067521</v>
+        <v>0.07890212841335756</v>
       </c>
       <c r="I15" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="16">
@@ -876,28 +875,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C16" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D16" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E16" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F16" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G16" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H16" t="n">
-        <v>0.06008794482067521</v>
+        <v>0.07890212841335756</v>
       </c>
       <c r="I16" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="17">
@@ -905,28 +904,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C17" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07891721960641043</v>
       </c>
       <c r="D17" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E17" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F17" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07891629781882403</v>
       </c>
       <c r="G17" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H17" t="n">
-        <v>0.06008791351248836</v>
+        <v>0.07890212835915958</v>
       </c>
       <c r="I17" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="18">
@@ -934,28 +933,28 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C18" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D18" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E18" t="n">
-        <v>0.06073701886393519</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F18" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G18" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H18" t="n">
-        <v>0.06008791293916189</v>
+        <v>0.0789021282779987</v>
       </c>
       <c r="I18" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="19">
@@ -963,28 +962,28 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C19" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D19" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E19" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F19" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G19" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H19" t="n">
-        <v>0.06008791293916189</v>
+        <v>0.0789021282779987</v>
       </c>
       <c r="I19" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="20">
@@ -992,28 +991,28 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C20" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D20" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E20" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890483850093846</v>
       </c>
       <c r="F20" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G20" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H20" t="n">
-        <v>0.06008791272563235</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I20" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="21">
@@ -1021,28 +1020,28 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C21" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D21" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E21" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F21" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G21" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H21" t="n">
-        <v>0.06008791272563235</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I21" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="22">
@@ -1050,28 +1049,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C22" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D22" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890767829743128</v>
       </c>
       <c r="E22" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F22" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G22" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H22" t="n">
-        <v>0.06008791256936866</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I22" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="23">
@@ -1079,28 +1078,28 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C23" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D23" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E23" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F23" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G23" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H23" t="n">
-        <v>0.06008791256936866</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I23" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="24">
@@ -1108,28 +1107,28 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C24" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D24" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E24" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F24" t="n">
-        <v>0.06008894098804901</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G24" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H24" t="n">
-        <v>0.06008791256936866</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I24" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="25">
@@ -1137,28 +1136,28 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C25" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D25" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E25" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F25" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G25" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H25" t="n">
-        <v>0.06008791254847922</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I25" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="26">
@@ -1166,28 +1165,28 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C26" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D26" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E26" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F26" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G26" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H26" t="n">
-        <v>0.06008791253555167</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I26" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="27">
@@ -1195,28 +1194,28 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890319315234148</v>
       </c>
       <c r="C27" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D27" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E27" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F27" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G27" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H27" t="n">
-        <v>0.06008791251433792</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I27" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="28">
@@ -1224,28 +1223,28 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890292411882832</v>
       </c>
       <c r="C28" t="n">
-        <v>0.06008842892403223</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D28" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E28" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F28" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G28" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H28" t="n">
-        <v>0.06008791251433792</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I28" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="29">
@@ -1253,28 +1252,28 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890292411882832</v>
       </c>
       <c r="C29" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D29" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E29" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F29" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G29" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H29" t="n">
-        <v>0.06008791251433792</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I29" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="30">
@@ -1282,28 +1281,28 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C30" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D30" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E30" t="n">
-        <v>0.06018355612703876</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F30" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G30" t="n">
-        <v>0.06008869114277009</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H30" t="n">
-        <v>0.06008791250469874</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I30" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="31">
@@ -1311,28 +1310,28 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C31" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D31" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E31" t="n">
-        <v>0.06013968373311566</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F31" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G31" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H31" t="n">
-        <v>0.06008791250469874</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I31" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="32">
@@ -1340,28 +1339,28 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C32" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D32" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E32" t="n">
-        <v>0.06009941418343663</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F32" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G32" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H32" t="n">
-        <v>0.06008791250469874</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I32" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="33">
@@ -1369,28 +1368,28 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C33" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D33" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E33" t="n">
-        <v>0.06009941418343663</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F33" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G33" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H33" t="n">
-        <v>0.06008791250312683</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I33" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="34">
@@ -1398,28 +1397,28 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C34" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D34" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E34" t="n">
-        <v>0.06009941418343663</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F34" t="n">
-        <v>0.06008871813698096</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G34" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H34" t="n">
-        <v>0.06008791250243394</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I34" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="35">
@@ -1427,28 +1426,28 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C35" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D35" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E35" t="n">
-        <v>0.06009941418343663</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F35" t="n">
-        <v>0.06008850149501168</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G35" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H35" t="n">
-        <v>0.06008791250241428</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I35" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="36">
@@ -1456,28 +1455,28 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>0.06008791276839962</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C36" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D36" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E36" t="n">
-        <v>0.06009941418343663</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F36" t="n">
-        <v>0.06008825377239523</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G36" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H36" t="n">
-        <v>0.06008791250241428</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I36" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="37">
@@ -1485,28 +1484,28 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C37" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D37" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E37" t="n">
-        <v>0.06008845697881401</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F37" t="n">
-        <v>0.06008825377239523</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G37" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H37" t="n">
-        <v>0.06008791250236965</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I37" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="38">
@@ -1514,28 +1513,28 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C38" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D38" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E38" t="n">
-        <v>0.06008845697881401</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F38" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G38" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H38" t="n">
-        <v>0.06008791250208938</v>
+        <v>0.07890207418518232</v>
       </c>
       <c r="I38" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="39">
@@ -1543,28 +1542,28 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C39" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D39" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E39" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F39" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G39" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H39" t="n">
-        <v>0.06008791250208938</v>
+        <v>0.07890207404124522</v>
       </c>
       <c r="I39" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="40">
@@ -1572,28 +1571,28 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D40" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E40" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F40" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G40" t="n">
-        <v>0.06008817847556249</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H40" t="n">
-        <v>0.06008791250208938</v>
+        <v>0.07890207404124522</v>
       </c>
       <c r="I40" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="41">
@@ -1601,28 +1600,28 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C41" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D41" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E41" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F41" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G41" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H41" t="n">
-        <v>0.06008791250208938</v>
+        <v>0.07890207404124522</v>
       </c>
       <c r="I41" t="n">
-        <v>0.06010232259186257</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="42">
@@ -1630,28 +1629,28 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890269187709881</v>
       </c>
       <c r="C42" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D42" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E42" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F42" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G42" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H42" t="n">
-        <v>0.0600879125020418</v>
+        <v>0.07890207336776091</v>
       </c>
       <c r="I42" t="n">
-        <v>0.06009419170379793</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="43">
@@ -1659,28 +1658,28 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>0.06008791266887335</v>
+        <v>0.07890267654744682</v>
       </c>
       <c r="C43" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D43" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.0789040840532873</v>
       </c>
       <c r="E43" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F43" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G43" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0600879125020418</v>
+        <v>0.07890207336776091</v>
       </c>
       <c r="I43" t="n">
-        <v>0.06009419170379793</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="44">
@@ -1688,28 +1687,28 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>0.06008791266707936</v>
+        <v>0.07890267654744682</v>
       </c>
       <c r="C44" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D44" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890386538573686</v>
       </c>
       <c r="E44" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F44" t="n">
-        <v>0.06008820371423982</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G44" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H44" t="n">
-        <v>0.0600879125020418</v>
+        <v>0.07890207336776091</v>
       </c>
       <c r="I44" t="n">
-        <v>0.06009419170379793</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="45">
@@ -1717,28 +1716,28 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>0.06008791266661043</v>
+        <v>0.07890267654744682</v>
       </c>
       <c r="C45" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D45" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890386538573686</v>
       </c>
       <c r="E45" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F45" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G45" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H45" t="n">
-        <v>0.0600879125020418</v>
+        <v>0.07890207336776091</v>
       </c>
       <c r="I45" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="46">
@@ -1746,28 +1745,28 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>0.06008791262345908</v>
+        <v>0.07890267654744682</v>
       </c>
       <c r="C46" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D46" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890386538573686</v>
       </c>
       <c r="E46" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F46" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G46" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H46" t="n">
-        <v>0.0600879125020418</v>
+        <v>0.07890207336776091</v>
       </c>
       <c r="I46" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="47">
@@ -1775,28 +1774,28 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>0.06008791262345908</v>
+        <v>0.07890267654744682</v>
       </c>
       <c r="C47" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D47" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890265416815881</v>
       </c>
       <c r="E47" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F47" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G47" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H47" t="n">
-        <v>0.0600879125020249</v>
+        <v>0.07890207336776091</v>
       </c>
       <c r="I47" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="48">
@@ -1804,28 +1803,28 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>0.06008791262345908</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C48" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D48" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890265416815881</v>
       </c>
       <c r="E48" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F48" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G48" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0600879125020249</v>
+        <v>0.07890207336046731</v>
       </c>
       <c r="I48" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="49">
@@ -1833,28 +1832,28 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>0.06008791258204844</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C49" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D49" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890265416815881</v>
       </c>
       <c r="E49" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F49" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G49" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H49" t="n">
-        <v>0.0600879125020249</v>
+        <v>0.07890207336046731</v>
       </c>
       <c r="I49" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="50">
@@ -1862,28 +1861,28 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>0.06008791258204844</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C50" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D50" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890265416815881</v>
       </c>
       <c r="E50" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F50" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890442779688002</v>
       </c>
       <c r="G50" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H50" t="n">
-        <v>0.0600879125020249</v>
+        <v>0.07890207336046731</v>
       </c>
       <c r="I50" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="51">
@@ -1891,28 +1890,28 @@
         <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>0.06008791258204844</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C51" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D51" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E51" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F51" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G51" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H51" t="n">
-        <v>0.0600879125020249</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I51" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="52">
@@ -1920,28 +1919,28 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>0.0600879125610946</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C52" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D52" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E52" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F52" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G52" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H52" t="n">
-        <v>0.06008791250184746</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I52" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="53">
@@ -1949,28 +1948,28 @@
         <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>0.0600879125610946</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C53" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D53" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E53" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F53" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G53" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H53" t="n">
-        <v>0.06008791250184557</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I53" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="54">
@@ -1978,28 +1977,28 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>0.0600879125610946</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C54" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D54" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E54" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F54" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G54" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H54" t="n">
-        <v>0.06008791250184557</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I54" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="55">
@@ -2007,28 +2006,28 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>0.06008791252841451</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C55" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D55" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E55" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F55" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G55" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H55" t="n">
-        <v>0.06008791250184557</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I55" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="56">
@@ -2036,28 +2035,28 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>0.06008791252841451</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C56" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D56" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E56" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F56" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G56" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H56" t="n">
-        <v>0.06008791250184557</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I56" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="57">
@@ -2065,28 +2064,28 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C57" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D57" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E57" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F57" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G57" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H57" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I57" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="58">
@@ -2094,28 +2093,28 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890246646149733</v>
       </c>
       <c r="C58" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D58" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E58" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F58" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G58" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H58" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I58" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="59">
@@ -2123,28 +2122,28 @@
         <v>58</v>
       </c>
       <c r="B59" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C59" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D59" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E59" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F59" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G59" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H59" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I59" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="60">
@@ -2152,28 +2151,28 @@
         <v>59</v>
       </c>
       <c r="B60" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C60" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D60" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E60" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F60" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G60" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H60" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I60" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="61">
@@ -2181,28 +2180,28 @@
         <v>60</v>
       </c>
       <c r="B61" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C61" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D61" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E61" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F61" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G61" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H61" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I61" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="62">
@@ -2210,28 +2209,28 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C62" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D62" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E62" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F62" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G62" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H62" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I62" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="63">
@@ -2239,28 +2238,28 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C63" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D63" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E63" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F63" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G63" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H63" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I63" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="64">
@@ -2268,28 +2267,28 @@
         <v>63</v>
       </c>
       <c r="B64" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C64" t="n">
-        <v>0.06008839523965438</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D64" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E64" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F64" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G64" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H64" t="n">
-        <v>0.06008791250184203</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I64" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="65">
@@ -2297,28 +2296,28 @@
         <v>64</v>
       </c>
       <c r="B65" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C65" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D65" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E65" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890369948924504</v>
       </c>
       <c r="F65" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G65" t="n">
-        <v>0.06008808437525144</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H65" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I65" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="66">
@@ -2326,28 +2325,28 @@
         <v>65</v>
       </c>
       <c r="B66" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890233944069125</v>
       </c>
       <c r="C66" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D66" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E66" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F66" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G66" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H66" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I66" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="67">
@@ -2355,28 +2354,28 @@
         <v>66</v>
       </c>
       <c r="B67" t="n">
-        <v>0.06008791250296631</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C67" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D67" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E67" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F67" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G67" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H67" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I67" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="68">
@@ -2384,28 +2383,28 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>0.06008791250233691</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C68" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D68" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E68" t="n">
-        <v>0.06008801600334657</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F68" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G68" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H68" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I68" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="69">
@@ -2413,28 +2412,28 @@
         <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>0.06008791250233691</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C69" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D69" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E69" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F69" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G69" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H69" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I69" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="70">
@@ -2442,28 +2441,28 @@
         <v>69</v>
       </c>
       <c r="B70" t="n">
-        <v>0.06008791250233405</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C70" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D70" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E70" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F70" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G70" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H70" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I70" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="71">
@@ -2471,28 +2470,28 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>0.06008791250233405</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C71" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D71" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E71" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F71" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890314293036939</v>
       </c>
       <c r="G71" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H71" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I71" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="72">
@@ -2500,28 +2499,28 @@
         <v>71</v>
       </c>
       <c r="B72" t="n">
-        <v>0.06008791250233405</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C72" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D72" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E72" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F72" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G72" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H72" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I72" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="73">
@@ -2529,28 +2528,28 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>0.06008791250233405</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C73" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D73" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E73" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F73" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G73" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H73" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I73" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="74">
@@ -2558,28 +2557,28 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>0.06008791250207917</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C74" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D74" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E74" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F74" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G74" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H74" t="n">
-        <v>0.06008791250183686</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I74" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="75">
@@ -2587,28 +2586,28 @@
         <v>74</v>
       </c>
       <c r="B75" t="n">
-        <v>0.06008791250207917</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C75" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D75" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E75" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F75" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G75" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H75" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I75" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="76">
@@ -2616,28 +2615,28 @@
         <v>75</v>
       </c>
       <c r="B76" t="n">
-        <v>0.06008791250207917</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C76" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D76" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E76" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F76" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G76" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H76" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I76" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="77">
@@ -2645,28 +2644,28 @@
         <v>76</v>
       </c>
       <c r="B77" t="n">
-        <v>0.06008791250207917</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C77" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D77" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E77" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F77" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G77" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H77" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I77" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="78">
@@ -2674,28 +2673,28 @@
         <v>77</v>
       </c>
       <c r="B78" t="n">
-        <v>0.06008791250207917</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C78" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D78" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E78" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F78" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G78" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H78" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I78" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="79">
@@ -2703,28 +2702,28 @@
         <v>78</v>
       </c>
       <c r="B79" t="n">
-        <v>0.06008791250207917</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C79" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D79" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E79" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F79" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G79" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H79" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I79" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="80">
@@ -2732,28 +2731,28 @@
         <v>79</v>
       </c>
       <c r="B80" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890229007603461</v>
       </c>
       <c r="C80" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D80" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E80" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F80" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G80" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H80" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I80" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="81">
@@ -2761,28 +2760,28 @@
         <v>80</v>
       </c>
       <c r="B81" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C81" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D81" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E81" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F81" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G81" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H81" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I81" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="82">
@@ -2790,28 +2789,28 @@
         <v>81</v>
       </c>
       <c r="B82" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C82" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D82" t="n">
-        <v>0.06008824301451486</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E82" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F82" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G82" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H82" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I82" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="83">
@@ -2819,28 +2818,28 @@
         <v>82</v>
       </c>
       <c r="B83" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C83" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D83" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E83" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F83" t="n">
-        <v>0.06008793556394845</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G83" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H83" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I83" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="84">
@@ -2848,28 +2847,28 @@
         <v>83</v>
       </c>
       <c r="B84" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C84" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D84" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E84" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F84" t="n">
-        <v>0.06008792155219173</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G84" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H84" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I84" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="85">
@@ -2877,28 +2876,28 @@
         <v>84</v>
       </c>
       <c r="B85" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C85" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D85" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E85" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F85" t="n">
-        <v>0.06008792155219173</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G85" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H85" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I85" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="86">
@@ -2906,28 +2905,28 @@
         <v>85</v>
       </c>
       <c r="B86" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C86" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D86" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E86" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F86" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G86" t="n">
-        <v>0.06008796363935772</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H86" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I86" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="87">
@@ -2935,28 +2934,28 @@
         <v>86</v>
       </c>
       <c r="B87" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C87" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D87" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E87" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F87" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G87" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H87" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I87" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="88">
@@ -2964,28 +2963,28 @@
         <v>87</v>
       </c>
       <c r="B88" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C88" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D88" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E88" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F88" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G88" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H88" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I88" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="89">
@@ -2993,28 +2992,28 @@
         <v>88</v>
       </c>
       <c r="B89" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C89" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D89" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E89" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F89" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G89" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H89" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I89" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="90">
@@ -3022,28 +3021,28 @@
         <v>89</v>
       </c>
       <c r="B90" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890222702575719</v>
       </c>
       <c r="C90" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D90" t="n">
-        <v>0.06008809419061413</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E90" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F90" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G90" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H90" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I90" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="91">
@@ -3051,28 +3050,28 @@
         <v>90</v>
       </c>
       <c r="B91" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890213613615932</v>
       </c>
       <c r="C91" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D91" t="n">
-        <v>0.06008800280640962</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E91" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F91" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G91" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H91" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I91" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="92">
@@ -3080,28 +3079,28 @@
         <v>91</v>
       </c>
       <c r="B92" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890213613615932</v>
       </c>
       <c r="C92" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D92" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E92" t="n">
-        <v>0.06008794331047626</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F92" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G92" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H92" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I92" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="93">
@@ -3109,28 +3108,28 @@
         <v>92</v>
       </c>
       <c r="B93" t="n">
-        <v>0.060087912502039</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C93" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D93" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E93" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F93" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G93" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H93" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207332087668</v>
       </c>
       <c r="I93" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="94">
@@ -3138,28 +3137,28 @@
         <v>93</v>
       </c>
       <c r="B94" t="n">
-        <v>0.06008791250201838</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C94" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D94" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E94" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F94" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G94" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H94" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I94" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="95">
@@ -3167,28 +3166,28 @@
         <v>94</v>
       </c>
       <c r="B95" t="n">
-        <v>0.06008791250201838</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C95" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D95" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890236714792212</v>
       </c>
       <c r="E95" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F95" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G95" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H95" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I95" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="96">
@@ -3196,28 +3195,28 @@
         <v>95</v>
       </c>
       <c r="B96" t="n">
-        <v>0.06008791250201838</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C96" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D96" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890233703440339</v>
       </c>
       <c r="E96" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F96" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G96" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H96" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I96" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="97">
@@ -3225,28 +3224,28 @@
         <v>96</v>
       </c>
       <c r="B97" t="n">
-        <v>0.0600879125020134</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C97" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D97" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890233703440339</v>
       </c>
       <c r="E97" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F97" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890290025145631</v>
       </c>
       <c r="G97" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H97" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I97" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="98">
@@ -3254,28 +3253,28 @@
         <v>97</v>
       </c>
       <c r="B98" t="n">
-        <v>0.0600879125020134</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C98" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D98" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890232337555525</v>
       </c>
       <c r="E98" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F98" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890277010904079</v>
       </c>
       <c r="G98" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H98" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I98" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="99">
@@ -3283,28 +3282,28 @@
         <v>98</v>
       </c>
       <c r="B99" t="n">
-        <v>0.0600879125020134</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C99" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D99" t="n">
-        <v>0.06008799002006221</v>
+        <v>0.07890229230281358</v>
       </c>
       <c r="E99" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F99" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890277010904079</v>
       </c>
       <c r="G99" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H99" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I99" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="100">
@@ -3312,28 +3311,28 @@
         <v>99</v>
       </c>
       <c r="B100" t="n">
-        <v>0.0600879125020134</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C100" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D100" t="n">
-        <v>0.06008794403749526</v>
+        <v>0.07890229230281358</v>
       </c>
       <c r="E100" t="n">
-        <v>0.06008792269155933</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F100" t="n">
-        <v>0.06008791908238273</v>
+        <v>0.07890277010904079</v>
       </c>
       <c r="G100" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H100" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I100" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
     <row r="101">
@@ -3341,28 +3340,28 @@
         <v>100</v>
       </c>
       <c r="B101" t="n">
-        <v>0.0600879125020134</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C101" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="D101" t="n">
-        <v>0.06008794403749526</v>
+        <v>0.07890229032410366</v>
       </c>
       <c r="E101" t="n">
-        <v>0.06008792261201259</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="F101" t="n">
-        <v>0.06008791662776609</v>
+        <v>0.07890277010904079</v>
       </c>
       <c r="G101" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="H101" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="I101" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890286120937849</v>
       </c>
     </row>
   </sheetData>
@@ -3423,22 +3422,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.06008791250183247</v>
+        <v>0.07890207331384931</v>
       </c>
       <c r="C2" t="n">
-        <v>0.003610557228827875</v>
+        <v>0.006225537173224051</v>
       </c>
       <c r="D2" t="n">
-        <v>3.008654356002808</v>
+        <v>5.687664031982422</v>
       </c>
       <c r="E2" t="n">
-        <v>19.57309838251803</v>
+        <v>14.67578635553511</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8266723714506453</v>
+        <v>0.9662188352978063</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7572723199750544</v>
+        <v>1.840007032491966</v>
       </c>
     </row>
     <row r="3">
@@ -3448,72 +3447,72 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0600879125020134</v>
+        <v>0.07890213110246531</v>
       </c>
       <c r="C3" t="n">
-        <v>0.003610557228849618</v>
+        <v>0.006225546292510624</v>
       </c>
       <c r="D3" t="n">
-        <v>4.671249628067017</v>
+        <v>14.9656445980072</v>
       </c>
       <c r="E3" t="n">
-        <v>18.79589423577081</v>
+        <v>14.39313370195358</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9289862698942818</v>
+        <v>1.274969342291042</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6214168676757164</v>
+        <v>1.286406683136417</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IGOA</t>
+          <t>VCS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.06008791662776609</v>
+        <v>0.07890229032410366</v>
       </c>
       <c r="C4" t="n">
-        <v>0.003610557724665368</v>
+        <v>0.006225571418389142</v>
       </c>
       <c r="D4" t="n">
-        <v>3.183907270431519</v>
+        <v>5.75753927230835</v>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>14.09806000239596</v>
       </c>
       <c r="F4" t="n">
-        <v>0.648477200636012</v>
+        <v>0.7084645383533422</v>
       </c>
       <c r="G4" t="n">
-        <v>1.007945534437748</v>
+        <v>1.815459188230969</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HGS</t>
+          <t>ESA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.06008792261201259</v>
+        <v>0.07890230141110996</v>
       </c>
       <c r="C5" t="n">
-        <v>0.003610558443827214</v>
+        <v>0.006225573167969645</v>
       </c>
       <c r="D5" t="n">
-        <v>3.013360023498535</v>
+        <v>6.384811162948608</v>
       </c>
       <c r="E5" t="n">
-        <v>13.74882000286159</v>
+        <v>16.86096234711786</v>
       </c>
       <c r="F5" t="n">
-        <v>0.188902390834387</v>
+        <v>0.9422401880468134</v>
       </c>
       <c r="G5" t="n">
-        <v>1.635086304619653</v>
+        <v>1.554703558565153</v>
       </c>
     </row>
     <row r="6">
@@ -3523,213 +3522,97 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06008793069314096</v>
+        <v>0.07890230867297976</v>
       </c>
       <c r="C6" t="n">
-        <v>0.003610559414983711</v>
+        <v>0.006225574313926177</v>
       </c>
       <c r="D6" t="n">
-        <v>3.129085063934326</v>
+        <v>5.923944473266602</v>
       </c>
       <c r="E6" t="n">
-        <v>18.97630079695606</v>
+        <v>16.83038400837917</v>
       </c>
       <c r="F6" t="n">
-        <v>1.029039449919565</v>
+        <v>1.408946562975902</v>
       </c>
       <c r="G6" t="n">
-        <v>0.571772252584033</v>
+        <v>0.907067072791683</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VCS</t>
+          <t>IGOA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.06008794403749526</v>
+        <v>0.07890277010904079</v>
       </c>
       <c r="C7" t="n">
-        <v>0.003610561018653162</v>
+        <v>0.00622564713088014</v>
       </c>
       <c r="D7" t="n">
-        <v>3.108911991119385</v>
+        <v>6.353922605514526</v>
       </c>
       <c r="E7" t="n">
-        <v>16.66897255366866</v>
+        <v>12.26982989535685</v>
       </c>
       <c r="F7" t="n">
-        <v>1.59231860750472</v>
+        <v>1.707723198300801</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2851648660414028</v>
+        <v>0.6009940201003026</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ESA</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.06008823159060829</v>
+        <v>0.07890286120937849</v>
       </c>
       <c r="C8" t="n">
-        <v>0.003610595575686576</v>
+        <v>0.006225661507026445</v>
       </c>
       <c r="D8" t="n">
-        <v>3.262387275695801</v>
+        <v>5.754862308502197</v>
       </c>
       <c r="E8" t="n">
-        <v>17.22809249790414</v>
+        <v>16.0846876795679</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4144810798115213</v>
+        <v>1.324120463209017</v>
       </c>
       <c r="G8" t="n">
-        <v>1.168664775805079</v>
+        <v>0.6666783458982248</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>HGS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.06008885430174732</v>
+        <v>0.07890305903640348</v>
       </c>
       <c r="C9" t="n">
-        <v>0.003610670411296617</v>
+        <v>0.006225692725302172</v>
       </c>
       <c r="D9" t="n">
-        <v>3.577211380004883</v>
+        <v>5.727043867111206</v>
       </c>
       <c r="E9" t="n">
-        <v>20</v>
+        <v>13.46088146982569</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8093001174680976</v>
+        <v>0.970972250123154</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8103425875536407</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>pop_size</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>max_iter</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>dimensions</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Kp_range</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>[1, 20]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>T1_range</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>[0.05, 2.0]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>T2_range</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>[0.05, 2.0]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>objective</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ITAE (odeint-based PSS optimization)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-05-26 08:51:10</t>
-        </is>
+        <v>1.134412318002246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>